<commit_message>
Update local settings and June 2026 sales summary
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/June_2026_Sales_Summary.xlsx
+++ b/June_2026_Sales_Summary.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_8EA35FE92E7CB7DD6FDE4D1C1B2F05D2972A5790" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4FB2485C-8955-4266-9BA1-291F1585F819}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="11_8EA35FE92E7CB7DD6FDE4D1C1B2F05D2972A5790" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A5C2398F-24CD-4316-890E-3E3CC542A5E6}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -13,6 +13,7 @@
     <sheet name="June 2026 - Ex Texas" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>

</xml_diff>